<commit_message>
Add GRN scan script with pagination + 80% zoom config
- New tests/m3/grn-scan.spec.js: Phase 3 inventory -> Phase 4 device scanning -> Phase 5 confirm GRN, with console pause for data verification
- New playwright.config.js: default config with --force-device-scale-factor=0.8 (80% zoom)
- InventoryViewPage: collectRowData loops through all pagination pages
- ConfirmGRNPage: selectAllRowsViaHeaderCheckbox loops through all pagination pages before Update M3
- Added pagination locators to ConfirmGRNLocators and InventoryViewLocators
- Added grn / grn:headed npm scripts to package.json

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/m3/po-numbers.xlsx
+++ b/data/m3/po-numbers.xlsx
@@ -389,93 +389,59 @@
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="1">
-        <v>1010047516</v>
+        <v>1010033472</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
-      <c r="A3" s="1">
-        <v>1010047517</v>
-      </c>
+      <c r="A3" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
-      <c r="A4" s="1">
-        <v>1010047519</v>
-      </c>
+      <c r="A4" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
-      <c r="A5" s="1">
-        <v>1010047521</v>
-      </c>
+      <c r="A5" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
-      <c r="A6" s="1">
-        <v>1010047520</v>
-      </c>
+      <c r="A6" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
-      <c r="A7" s="1">
-        <v>1010047518</v>
-      </c>
+      <c r="A7" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
-      <c r="A8" s="1">
-        <v>1010047522</v>
-      </c>
+      <c r="A8" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
-      <c r="A9" s="1">
-        <v>1010047523</v>
-      </c>
+      <c r="A9" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
-      <c r="A10" s="1">
-        <v>1010047525</v>
-      </c>
+      <c r="A10" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
-      <c r="A11" s="1">
-        <v>1010047527</v>
-      </c>
+      <c r="A11" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
-      <c r="A12" s="1">
-        <v>1010047526</v>
-      </c>
+      <c r="A12" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
-      <c r="A13" s="1">
-        <v>1010047524</v>
-      </c>
+      <c r="A13" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
-      <c r="A14" s="1">
-        <v>1010047530</v>
-      </c>
+      <c r="A14" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
-      <c r="A15" s="1">
-        <v>1010047529</v>
-      </c>
+      <c r="A15" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
-      <c r="A16" s="1">
-        <v>1010047528</v>
-      </c>
+      <c r="A16" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5">
-      <c r="A17" s="1">
-        <v>1010047533</v>
-      </c>
+      <c r="A17" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
-      <c r="A18" s="1">
-        <v>1010047532</v>
-      </c>
+      <c r="A18" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="19.5">
-      <c r="A19" s="1">
-        <v>1010047531</v>
-      </c>
+      <c r="A19" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="19.5">
       <c r="A20" s="1"/>

</xml_diff>